<commit_message>
v2.2: revision publicaciones may-jun26 (14 tickers) + updates feed, deltas strip, calendario est., history ±1σ, backtest drawdown, mobile sidebar
</commit_message>
<xml_diff>
--- a/data/raw/watchlist_ratings.xlsx
+++ b/data/raw/watchlist_ratings.xlsx
@@ -14064,9 +14064,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BP65"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5703125" defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -14118,7 +14118,7 @@
     <col min="67" max="67" width="11.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:68" ht="27.75" customHeight="1" ns3:dyDescent="0.25">
       <c r="A1" s="100" t="s">
         <v>0</v>
       </c>
@@ -14171,7 +14171,7 @@
       <c r="AV1" s="96"/>
       <c r="AW1" s="96"/>
     </row>
-    <row r="2" spans="1:68" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:68" ht="21.75" customHeight="1" ns3:dyDescent="0.25">
       <c r="A2" s="103" t="s">
         <v>1</v>
       </c>
@@ -14257,7 +14257,7 @@
       <c r="BO2" s="96"/>
       <c r="BP2" s="96"/>
     </row>
-    <row r="3" spans="1:68" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:68" ht="45" customHeight="1" ns3:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>9</v>
       </c>
@@ -14461,7 +14461,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A4" s="86" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
@@ -14683,17 +14683,23 @@
         <f t="shared" ref="BM4:BM35" ca="1" si="20">(BK4/G4)^(1/4)-1</f>
         <v>0.34329692568943093</v>
       </c>
-      <c r="BN4" s="93" t="s">
-        <v>81</v>
-      </c>
-      <c r="BO4" s="93" t="s">
-        <v>82</v>
-      </c>
-      <c r="BP4" s="93" t="s">
-        <v>83</v>
+      <c r="BN4" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="BO4" t="inlineStr">
+        <is>
+          <t>03/06/2026</t>
+        </is>
+      </c>
+      <c r="BP4" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
       </c>
     </row>
-    <row r="5" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A5" s="86" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
@@ -14925,7 +14931,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="6" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A6" s="86" t="e" vm="3">
         <v>#VALUE!</v>
       </c>
@@ -15157,7 +15163,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="7" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A7" s="86" t="e" vm="4">
         <v>#VALUE!</v>
       </c>
@@ -15379,17 +15385,23 @@
         <f t="shared" ca="1" si="20"/>
         <v>0.25007229949436627</v>
       </c>
-      <c r="BN7" s="93" t="s">
-        <v>81</v>
-      </c>
-      <c r="BO7" s="94" t="s">
-        <v>98</v>
-      </c>
-      <c r="BP7" s="93" t="s">
-        <v>99</v>
+      <c r="BN7" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="BO7" t="inlineStr">
+        <is>
+          <t>14/05/2026</t>
+        </is>
+      </c>
+      <c r="BP7" t="inlineStr">
+        <is>
+          <t>13/08/2026</t>
+        </is>
       </c>
     </row>
-    <row r="8" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A8" s="86" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
@@ -15611,17 +15623,23 @@
         <f t="shared" ca="1" si="20"/>
         <v>-1.6089199691735612E-2</v>
       </c>
-      <c r="BN8" s="93" t="s">
-        <v>81</v>
-      </c>
-      <c r="BO8" s="93" t="s">
-        <v>103</v>
-      </c>
-      <c r="BP8" s="93" t="s">
-        <v>104</v>
+      <c r="BN8" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="BO8" t="inlineStr">
+        <is>
+          <t>28/05/2026</t>
+        </is>
+      </c>
+      <c r="BP8" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
       </c>
     </row>
-    <row r="9" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A9" s="86" t="e" vm="6">
         <v>#VALUE!</v>
       </c>
@@ -15843,17 +15861,23 @@
         <f t="shared" ca="1" si="20"/>
         <v>0.22845688983290469</v>
       </c>
-      <c r="BN9" s="93" t="s">
-        <v>81</v>
-      </c>
-      <c r="BO9" s="93" t="s">
-        <v>107</v>
-      </c>
-      <c r="BP9" s="93" t="s">
-        <v>108</v>
+      <c r="BN9" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="BO9" t="inlineStr">
+        <is>
+          <t>03/06/2026</t>
+        </is>
+      </c>
+      <c r="BP9" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
       </c>
     </row>
-    <row r="10" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A10" s="86" t="e" vm="7">
         <v>#VALUE!</v>
       </c>
@@ -16085,7 +16109,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="11" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A11" s="86" t="e" vm="8">
         <v>#VALUE!</v>
       </c>
@@ -16307,17 +16331,23 @@
         <f t="shared" ca="1" si="20"/>
         <v>0.23909386335572558</v>
       </c>
-      <c r="BN11" s="93" t="s">
-        <v>81</v>
-      </c>
-      <c r="BO11" s="93" t="s">
-        <v>118</v>
-      </c>
-      <c r="BP11" s="93" t="s">
-        <v>104</v>
+      <c r="BN11" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="BO11" t="inlineStr">
+        <is>
+          <t>28/05/2026</t>
+        </is>
+      </c>
+      <c r="BP11" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
       </c>
     </row>
-    <row r="12" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A12" s="86" t="e" vm="9">
         <v>#VALUE!</v>
       </c>
@@ -16549,7 +16579,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="13" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A13" s="86" t="e" vm="10">
         <v>#VALUE!</v>
       </c>
@@ -16781,7 +16811,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="14" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A14" s="86" t="e" vm="11">
         <v>#VALUE!</v>
       </c>
@@ -17013,7 +17043,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="15" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A15" s="86" t="e" vm="12">
         <v>#VALUE!</v>
       </c>
@@ -17235,17 +17265,23 @@
         <f t="shared" ca="1" si="20"/>
         <v>0.16540754702958971</v>
       </c>
-      <c r="BN15" s="93" t="s">
-        <v>81</v>
-      </c>
-      <c r="BO15" s="93" t="s">
-        <v>134</v>
-      </c>
-      <c r="BP15" s="93" t="s">
-        <v>108</v>
+      <c r="BN15" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="BO15" t="inlineStr">
+        <is>
+          <t>09/06/2026</t>
+        </is>
+      </c>
+      <c r="BP15" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
       </c>
     </row>
-    <row r="16" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A16" s="86" t="e" vm="13">
         <v>#VALUE!</v>
       </c>
@@ -17477,7 +17513,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="17" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A17" s="86" t="e" vm="14">
         <v>#VALUE!</v>
       </c>
@@ -17709,7 +17745,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="18" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A18" s="86" t="e" vm="15">
         <v>#VALUE!</v>
       </c>
@@ -17941,7 +17977,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="19" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A19" s="86" t="e" vm="16">
         <v>#VALUE!</v>
       </c>
@@ -18173,7 +18209,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="20" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A20" s="86" t="e" vm="17">
         <v>#VALUE!</v>
       </c>
@@ -18395,17 +18431,23 @@
         <f t="shared" ca="1" si="20"/>
         <v>0.35157533189574863</v>
       </c>
-      <c r="BN20" s="93" t="s">
-        <v>81</v>
-      </c>
-      <c r="BO20" s="93" t="s">
-        <v>123</v>
-      </c>
-      <c r="BP20" s="93" t="s">
-        <v>104</v>
+      <c r="BN20" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="BO20" t="inlineStr">
+        <is>
+          <t>28/05/2026</t>
+        </is>
+      </c>
+      <c r="BP20" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
       </c>
     </row>
-    <row r="21" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A21" s="86" t="e" vm="18">
         <v>#VALUE!</v>
       </c>
@@ -18637,7 +18679,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="22" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A22" s="86" t="e" vm="19">
         <v>#VALUE!</v>
       </c>
@@ -18869,7 +18911,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="23" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A23" s="86" t="e" vm="20">
         <v>#VALUE!</v>
       </c>
@@ -19091,17 +19133,23 @@
         <f t="shared" ca="1" si="20"/>
         <v>6.3700785282530648E-2</v>
       </c>
-      <c r="BN23" s="93" t="s">
-        <v>81</v>
-      </c>
-      <c r="BO23" s="93" t="s">
-        <v>123</v>
-      </c>
-      <c r="BP23" s="93" t="s">
-        <v>99</v>
+      <c r="BN23" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="BO23" t="inlineStr">
+        <is>
+          <t>14/05/2026</t>
+        </is>
+      </c>
+      <c r="BP23" t="inlineStr">
+        <is>
+          <t>13/08/2026</t>
+        </is>
       </c>
     </row>
-    <row r="24" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A24" s="86" t="e" vm="21">
         <v>#VALUE!</v>
       </c>
@@ -19333,7 +19381,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="25" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A25" s="86" t="e" vm="22">
         <v>#VALUE!</v>
       </c>
@@ -19565,7 +19613,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="26" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A26" s="86" t="e" vm="23">
         <v>#VALUE!</v>
       </c>
@@ -19797,7 +19845,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="27" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A27" s="86" t="e" vm="24">
         <v>#VALUE!</v>
       </c>
@@ -20029,7 +20077,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="28" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A28" s="86" t="e" vm="25">
         <v>#VALUE!</v>
       </c>
@@ -20261,7 +20309,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="29" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A29" s="86" t="e" vm="26">
         <v>#VALUE!</v>
       </c>
@@ -20493,7 +20541,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="30" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A30" s="86" t="e" vm="27">
         <v>#VALUE!</v>
       </c>
@@ -20725,7 +20773,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="31" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A31" s="86" t="e" vm="28">
         <v>#VALUE!</v>
       </c>
@@ -20947,17 +20995,23 @@
         <f t="shared" ca="1" si="20"/>
         <v>-7.0078191617545804E-2</v>
       </c>
-      <c r="BN31" s="93" t="s">
-        <v>81</v>
-      </c>
-      <c r="BO31" s="93" t="s">
-        <v>186</v>
-      </c>
-      <c r="BP31" s="93" t="s">
-        <v>187</v>
+      <c r="BN31" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="BO31" t="inlineStr">
+        <is>
+          <t>03/06/2026</t>
+        </is>
+      </c>
+      <c r="BP31" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
       </c>
     </row>
-    <row r="32" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A32" s="86" t="e" vm="29">
         <v>#VALUE!</v>
       </c>
@@ -21189,7 +21243,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="33" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A33" s="86" t="e" vm="30">
         <v>#VALUE!</v>
       </c>
@@ -21421,7 +21475,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="34" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A34" s="86" t="e" vm="31">
         <v>#VALUE!</v>
       </c>
@@ -21653,7 +21707,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="35" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A35" s="86" t="e" vm="32">
         <v>#VALUE!</v>
       </c>
@@ -21885,7 +21939,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="36" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A36" s="86" t="e" vm="33">
         <v>#VALUE!</v>
       </c>
@@ -22107,17 +22161,23 @@
         <f t="shared" ref="BM36:BM65" ca="1" si="44">(BK36/G36)^(1/4)-1</f>
         <v>0.19198564331280221</v>
       </c>
-      <c r="BN36" s="93" t="s">
-        <v>81</v>
-      </c>
-      <c r="BO36" s="93" t="s">
-        <v>206</v>
-      </c>
-      <c r="BP36" s="93" t="s">
-        <v>207</v>
+      <c r="BN36" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="BO36" t="inlineStr">
+        <is>
+          <t>11/05/2026</t>
+        </is>
+      </c>
+      <c r="BP36" t="inlineStr">
+        <is>
+          <t>27/07/2026</t>
+        </is>
       </c>
     </row>
-    <row r="37" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A37" s="86" t="e" vm="34">
         <v>#VALUE!</v>
       </c>
@@ -22349,7 +22409,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="38" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A38" s="86" t="e" vm="35">
         <v>#VALUE!</v>
       </c>
@@ -22571,17 +22631,23 @@
         <f t="shared" ca="1" si="44"/>
         <v>7.7459442978258242E-2</v>
       </c>
-      <c r="BN38" s="93" t="s">
-        <v>81</v>
-      </c>
-      <c r="BO38" s="93" t="s">
-        <v>213</v>
-      </c>
-      <c r="BP38" s="93" t="s">
-        <v>214</v>
+      <c r="BN38" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="BO38" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="BP38" t="inlineStr">
+        <is>
+          <t>26/08/2026</t>
+        </is>
       </c>
     </row>
-    <row r="39" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A39" s="86" t="e" vm="36">
         <v>#VALUE!</v>
       </c>
@@ -22813,7 +22879,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="40" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A40" s="86" t="e" vm="37">
         <v>#VALUE!</v>
       </c>
@@ -23045,7 +23111,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="41" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A41" s="86" t="e" vm="38">
         <v>#VALUE!</v>
       </c>
@@ -23277,7 +23343,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="42" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A42" s="86" t="e" vm="39">
         <v>#VALUE!</v>
       </c>
@@ -23509,7 +23575,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="43" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A43" s="86" t="e" vm="40">
         <v>#VALUE!</v>
       </c>
@@ -23741,7 +23807,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="44" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A44" s="86" t="e" vm="41">
         <v>#VALUE!</v>
       </c>
@@ -23973,7 +24039,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="45" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A45" s="86" t="e" vm="42">
         <v>#VALUE!</v>
       </c>
@@ -24205,7 +24271,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="46" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A46" s="86" t="e" vm="43">
         <v>#VALUE!</v>
       </c>
@@ -24437,7 +24503,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="47" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A47" s="86" t="e" vm="44">
         <v>#VALUE!</v>
       </c>
@@ -24669,7 +24735,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="48" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A48" s="86" t="e" vm="45">
         <v>#VALUE!</v>
       </c>
@@ -24901,7 +24967,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="49" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A49" s="86" t="e" vm="46">
         <v>#VALUE!</v>
       </c>
@@ -25133,7 +25199,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="50" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A50" s="86" t="e" vm="47">
         <v>#VALUE!</v>
       </c>
@@ -25367,7 +25433,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="51" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A51" s="86" t="e" vm="48">
         <v>#VALUE!</v>
       </c>
@@ -25599,7 +25665,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="52" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A52" s="86" t="e" vm="49">
         <v>#VALUE!</v>
       </c>
@@ -25831,7 +25897,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="53" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A53" s="86" t="e" vm="50">
         <v>#VALUE!</v>
       </c>
@@ -26063,7 +26129,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="54" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A54" s="86" t="e" vm="51">
         <v>#VALUE!</v>
       </c>
@@ -26285,17 +26351,23 @@
         <f t="shared" ca="1" si="44"/>
         <v>-2.1023309776532217E-3</v>
       </c>
-      <c r="BN54" s="93" t="s">
-        <v>81</v>
-      </c>
-      <c r="BO54" s="93" t="s">
-        <v>261</v>
-      </c>
-      <c r="BP54" s="93" t="s">
-        <v>83</v>
+      <c r="BN54" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="BO54" t="inlineStr">
+        <is>
+          <t>28/05/2026</t>
+        </is>
+      </c>
+      <c r="BP54" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
       </c>
     </row>
-    <row r="55" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A55" s="86" t="e" vm="52">
         <v>#VALUE!</v>
       </c>
@@ -26527,7 +26599,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="56" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A56" s="86" t="e" vm="53">
         <v>#VALUE!</v>
       </c>
@@ -26759,7 +26831,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="57" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A57" s="86" t="e" vm="54">
         <v>#VALUE!</v>
       </c>
@@ -26991,7 +27063,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="58" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A58" s="86" t="e" vm="55">
         <v>#VALUE!</v>
       </c>
@@ -27213,17 +27285,23 @@
         <f t="shared" ca="1" si="44"/>
         <v>0.26657523111483949</v>
       </c>
-      <c r="BN58" s="93" t="s">
-        <v>81</v>
-      </c>
-      <c r="BO58" s="93" t="s">
-        <v>118</v>
-      </c>
-      <c r="BP58" s="93" t="s">
-        <v>207</v>
+      <c r="BN58" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="BO58" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="BP58" t="inlineStr">
+        <is>
+          <t>06/08/2026</t>
+        </is>
       </c>
     </row>
-    <row r="59" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A59" s="86" t="e" vm="56">
         <v>#VALUE!</v>
       </c>
@@ -27455,7 +27533,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="60" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A60" s="86" t="e" vm="57">
         <v>#VALUE!</v>
       </c>
@@ -27687,7 +27765,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="61" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A61" s="86" t="e" vm="58">
         <v>#VALUE!</v>
       </c>
@@ -27921,7 +27999,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="62" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A62" s="86" t="e" vm="59">
         <v>#VALUE!</v>
       </c>
@@ -28143,17 +28221,23 @@
         <f t="shared" ca="1" si="44"/>
         <v>0.1042738829072658</v>
       </c>
-      <c r="BN62" s="93" t="s">
-        <v>81</v>
-      </c>
-      <c r="BO62" s="94" t="s">
-        <v>275</v>
-      </c>
-      <c r="BP62" s="93" t="s">
-        <v>276</v>
+      <c r="BN62" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="BO62" t="inlineStr">
+        <is>
+          <t>14/05/2026</t>
+        </is>
+      </c>
+      <c r="BP62" t="inlineStr">
+        <is>
+          <t>02/07/2026</t>
+        </is>
       </c>
     </row>
-    <row r="63" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A63" s="86" t="e" vm="60">
         <v>#VALUE!</v>
       </c>
@@ -28385,7 +28469,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="64" spans="1:68" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:68" ht="15" customHeight="1" ns3:dyDescent="0.25">
       <c r="A64" s="86" t="e" vm="61">
         <v>#VALUE!</v>
       </c>
@@ -28617,7 +28701,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="65" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:68" ns3:dyDescent="0.25">
       <c r="A65" s="86" t="e" vm="62">
         <v>#VALUE!</v>
       </c>
@@ -28858,7 +28942,7 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <legacyDrawing r:id="rId1"/>
+  <legacyDrawing ns4:id="rId1"/>
 </worksheet>
 </file>
 
@@ -32970,9 +33054,9 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27.85546875" customWidth="1"/>
@@ -32980,7 +33064,7 @@
     <col min="5" max="5" width="192.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ns3:dyDescent="0.25">
       <c r="A1" t="s">
         <v>358</v>
       </c>
@@ -32997,7 +33081,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ns3:dyDescent="0.25">
       <c r="A2" t="s">
         <v>431</v>
       </c>
@@ -33014,7 +33098,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ns3:dyDescent="0.25">
       <c r="A3" t="s">
         <v>396</v>
       </c>
@@ -33031,7 +33115,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ns3:dyDescent="0.25">
       <c r="A4" t="s">
         <v>438</v>
       </c>
@@ -33048,7 +33132,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ns3:dyDescent="0.25">
       <c r="A5" t="s">
         <v>442</v>
       </c>
@@ -33065,7 +33149,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ns3:dyDescent="0.25">
       <c r="A6" t="s">
         <v>282</v>
       </c>
@@ -33080,6 +33164,384 @@
       </c>
       <c r="E6" t="s">
         <v>448</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BN Última actualización; BO Últimos resultados; BP Próximos resultados (est.)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Q1 FY27 press release + CNBC (20/05/2026)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Q1 FY27: rev $81.6B (+85%), Data Center $75.2B (+92%), EPS adj $1.87 beat; guía Q2 $91B; dividendo x25 a $0.25/trim. Vigilar digestión de expectativas (acción cayó pese al beat).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BN Última actualización; BO Últimos resultados; BP Próximos resultados (est.)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Q1 FY27 press release + transcript (03/06/2026)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Q1 FY27: ARR $5.51B, NNARR $256M (+32%), FCF $469M récord; sube guía NNARR FY27 +$50M; split 4:1 (jul). AIDR ARR +250% QoQ. Tesis de plataforma intacta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>VEEV</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BN Última actualización; BO Últimos resultados; BP Próximos resultados (est.)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Q1 FY27 press release + IR (03/06/2026)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Q1 FY27: rev $882.9M (+16%), subs +15%, EPS adj $2.24 beat; sube guía FY27. Pivot estratégico a AI agents (Vault CRM 150+ live). Vigilar ejecución Veeva AI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>BN Última actualización; BO Últimos resultados; BP Próximos resultados (est.)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Q3 FY26 press release (28/05/2026)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Q3 FY26: ventas $69.2B (+11.6%), comps +9.8% (+6.6% adj), EPS $4.93 (+15%), e-comm +21.5%, renovación US/CA 92.2%. Calidad operativa intacta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>BN Última actualización; BO Últimos resultados; BP Próximos resultados (est.)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Q3 FY26 press release (28/05/2026)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Q3 FY26: rev $850.5M (+25%), ARR $3.525B (+25%), NNARR $166M, margen op. non-GAAP récord 23%; guía FY26 ARR ~$3.74B (+24%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>BN Última actualización; BO Últimos resultados; BP Próximos resultados (est.)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Q1 FY27 press release (28/05/2026)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Q1 FY27: aceleración rev +21% ($277M), ARR $1.163B (+23%), NNARR récord $44M (+55%), margen op. +550bps a 4%. Inflexión crecimiento+rentabilidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ITX</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>BN Última actualización; BO Últimos resultados; BP Próximos resultados (est.)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Q1 2026 results + IR (09/06/2026)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Q1: ventas €8.75B (+5.8%; +8.8% cc), margen bruto 61.2% (+67bps), BN €1.4B (+5.4%); 1may-1jun +11.5% vs ~8% esperado; caja neta €10.8B. Momentum fuerte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>DNP</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>BN Última actualización; BO Últimos resultados; BP Próximos resultados (est.)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Q1 2026 report (14/05/2026)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Q1: rev PLN 8.9B (+14.8%), LFL +4.4%, EBITDA beat consenso +9%; 62 tiendas nuevas; margen EBITDA 6.7% (-50bps). Acción +13.7% el día.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BN</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BN Última actualización; BO Últimos resultados; BP Próximos resultados (est.)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Q1 2026 press release (14/05/2026)</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Q1: DE pre-realizaciones $0.59/sh (+7%), FRE +11%, capital fee-bearing +12%; $1B+ recompras YTD; avanza combinación BN+BNT. Tesis compounding intacta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>KSPI</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BN Última actualización; BO Últimos resultados; BP Próximos resultados (est.)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1Q 2026 results + transcript (11/05/2026)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Q1: rev +31% (KZT1.1T), GMV e-comm +41%, pero net income -1% (KZT252B); div KZT850/ADS (payout 64%); amortizó $600M notes. Vigilar compresión de márgenes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>EVD</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BN Última actualización; BO Últimos resultados; BP Próximos resultados (est.)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Q1 2026 results (28/05/2026)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Q1: rev €630M (+23%), aEBITDA €119M (+18.5%); Live Ent +38.3%; EPS €0.66 (+38%). Guidance reafirmado; ticketing algo débil por cambio de partner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>DSGX</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>BN Última actualización; BO Últimos resultados; BP Próximos resultados (est.)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Q1 FY27 press release (03/06/2026)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Q1 FY27: rev $193.6M (+15%), aEBITDA récord, net income $48.5M. Récords en márgenes y cash flow pese a mercado freight débil.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>WOSG</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BN Última actualización; BO Últimos resultados</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>FY26 Trading Update RNS (14/05/2026)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>FY26 (53 sem): rev récord £1.83B (+13% cc); US +24% ($1.24B, &gt;50% grupo); aEBIT £152-155M sobre guía; FY27 +5-10% cc. Resultados completos 02/07.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CELH</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BN Última actualización; BO Últimos resultados; BP Próximos resultados (est.)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Q1 2026 press release (07/05/2026)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Q1: rev $782.6M (+138% con Alani Nu/Rockstar), EPS $0.41 beat; cuota ~20.9%; margen bruto 48.3% (-400bps por mix adquisiciones). Vigilar integración.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
watchlist: multiplos de salida de Brookfield a 17,5-25
</commit_message>
<xml_diff>
--- a/data/raw/watchlist_ratings.xlsx
+++ b/data/raw/watchlist_ratings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roger\Cosas Roger\BOLSA E INVERSIÓN\repos\watchlist-dashboard\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FE73480-7667-4FE2-A271-F657789D3504}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18D54772-2AA0-4AD2-AA0F-0DB6FD9DACA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5876,155 +5876,33 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="44" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="40" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="23" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="4" fontId="28" fillId="40" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="34" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="20" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="23" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="28" fillId="40" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="37" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="30" fillId="37" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="28" fillId="40" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="30" fillId="37" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="39" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="25" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="29" fillId="25" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="23" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="33" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="42" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="15" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="29" fillId="25" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="4" fontId="29" fillId="25" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="15" fillId="43" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="32" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="19" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="16" fillId="23" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="22" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="29" fillId="25" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="29" fillId="25" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -6042,14 +5920,136 @@
     <xf numFmtId="0" fontId="15" fillId="41" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="34" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="19" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="40" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="16" fillId="23" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="23" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="22" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="33" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="42" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="43" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="32" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="37" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="30" fillId="37" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="28" fillId="40" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="30" fillId="37" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="39" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="23" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="44" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="40" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="23" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="28" fillId="40" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="20" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6848,7 +6848,7 @@
                   <c:v>0.27406080160124957</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.24224417295338063</c:v>
+                  <c:v>0.28381894079882097</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1.9692117436700851E-2</c:v>
@@ -17059,26 +17059,26 @@
         <v>0.12993869883637732</v>
       </c>
       <c r="BH7" s="24">
-        <v>13</v>
+        <v>17.5</v>
       </c>
       <c r="BI7" s="24">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="BJ7" s="25">
         <f t="shared" ca="1" si="17"/>
-        <v>33.104736501877106</v>
+        <v>45.66736611995114</v>
       </c>
       <c r="BK7" s="25">
         <f t="shared" ca="1" si="18"/>
-        <v>99.279542724768191</v>
+        <v>113.25229463500978</v>
       </c>
       <c r="BL7" s="23">
         <f t="shared" ca="1" si="19"/>
-        <v>-4.5069756479004019E-2</v>
+        <v>1.8391612561389437E-2</v>
       </c>
       <c r="BM7" s="23">
         <f t="shared" ca="1" si="20"/>
-        <v>0.24224417295338063</v>
+        <v>0.28381894079882097</v>
       </c>
       <c r="BN7" s="97">
         <v>46256</v>
@@ -32360,7 +32360,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:47" ht="45" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="112" t="s">
+      <c r="A1" s="168" t="s">
         <v>257</v>
       </c>
       <c r="B1" s="101"/>
@@ -32382,130 +32382,130 @@
       <c r="R1" s="32"/>
     </row>
     <row r="2" spans="1:47" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="129" t="s">
+      <c r="A2" s="156" t="s">
         <v>258</v>
       </c>
-      <c r="B2" s="130"/>
-      <c r="C2" s="130"/>
-      <c r="D2" s="130"/>
-      <c r="E2" s="130"/>
-      <c r="F2" s="130"/>
-      <c r="G2" s="130"/>
-      <c r="H2" s="130"/>
-      <c r="I2" s="130"/>
-      <c r="J2" s="130"/>
-      <c r="K2" s="130"/>
-      <c r="L2" s="130"/>
+      <c r="B2" s="157"/>
+      <c r="C2" s="157"/>
+      <c r="D2" s="157"/>
+      <c r="E2" s="157"/>
+      <c r="F2" s="157"/>
+      <c r="G2" s="157"/>
+      <c r="H2" s="157"/>
+      <c r="I2" s="157"/>
+      <c r="J2" s="157"/>
+      <c r="K2" s="157"/>
+      <c r="L2" s="157"/>
     </row>
     <row r="3" spans="1:47" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="135" t="s">
+      <c r="A3" s="161" t="s">
         <v>259</v>
       </c>
-      <c r="B3" s="124"/>
-      <c r="C3" s="156" t="s">
+      <c r="B3" s="129"/>
+      <c r="C3" s="128" t="s">
         <v>260</v>
       </c>
-      <c r="D3" s="124"/>
-      <c r="E3" s="157" t="s">
+      <c r="D3" s="129"/>
+      <c r="E3" s="130" t="s">
         <v>261</v>
       </c>
-      <c r="F3" s="124"/>
-      <c r="G3" s="123" t="s">
+      <c r="F3" s="129"/>
+      <c r="G3" s="176" t="s">
         <v>262</v>
       </c>
-      <c r="H3" s="124"/>
-      <c r="I3" s="125" t="s">
+      <c r="H3" s="129"/>
+      <c r="I3" s="177" t="s">
         <v>263</v>
       </c>
-      <c r="J3" s="124"/>
-      <c r="K3" s="161" t="s">
+      <c r="J3" s="129"/>
+      <c r="K3" s="140" t="s">
         <v>264</v>
       </c>
-      <c r="L3" s="162"/>
+      <c r="L3" s="141"/>
     </row>
     <row r="4" spans="1:47" ht="49.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="142">
+      <c r="A4" s="165">
         <f ca="1">COUNTA('Watchlist Ratings'!B4:B71)</f>
         <v>68</v>
       </c>
-      <c r="B4" s="127"/>
-      <c r="C4" s="158">
+      <c r="B4" s="135"/>
+      <c r="C4" s="136">
         <f>ROUND(AVERAGE('Watchlist Ratings'!AN4:AN71),2)</f>
         <v>5.98</v>
       </c>
-      <c r="D4" s="127"/>
-      <c r="E4" s="128" t="str">
+      <c r="D4" s="135"/>
+      <c r="E4" s="137" t="str">
         <f>TEXT(AVERAGE('Watchlist Ratings'!BC4:BC71),"0.0%")</f>
         <v>20.9%</v>
       </c>
-      <c r="F4" s="127"/>
-      <c r="G4" s="128" t="str">
+      <c r="F4" s="135"/>
+      <c r="G4" s="137" t="str">
         <f ca="1">TEXT(AVERAGE('Watchlist Ratings'!AW4:AW71),"0.0x")</f>
         <v>37.5x</v>
       </c>
-      <c r="H4" s="127"/>
-      <c r="I4" s="128">
+      <c r="H4" s="135"/>
+      <c r="I4" s="137">
         <f ca="1">COUNTIF('Watchlist Ratings'!BM4:BM71,"&gt;0")</f>
         <v>58</v>
       </c>
-      <c r="J4" s="127"/>
-      <c r="K4" s="113">
+      <c r="J4" s="135"/>
+      <c r="K4" s="169">
         <f>COUNTIF('Watchlist Ratings'!AN4:AN71,"&gt;7.5")</f>
         <v>16</v>
       </c>
-      <c r="L4" s="114"/>
+      <c r="L4" s="143"/>
     </row>
     <row r="5" spans="1:47" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="138" t="s">
+      <c r="A5" s="163" t="s">
         <v>265</v>
       </c>
-      <c r="B5" s="127"/>
-      <c r="C5" s="126" t="s">
+      <c r="B5" s="135"/>
+      <c r="C5" s="134" t="s">
         <v>266</v>
       </c>
-      <c r="D5" s="127"/>
-      <c r="E5" s="126" t="s">
+      <c r="D5" s="135"/>
+      <c r="E5" s="134" t="s">
         <v>267</v>
       </c>
-      <c r="F5" s="127"/>
-      <c r="G5" s="126" t="s">
+      <c r="F5" s="135"/>
+      <c r="G5" s="134" t="s">
         <v>268</v>
       </c>
-      <c r="H5" s="127"/>
-      <c r="I5" s="126" t="s">
+      <c r="H5" s="135"/>
+      <c r="I5" s="134" t="s">
         <v>269</v>
       </c>
-      <c r="J5" s="127"/>
-      <c r="K5" s="163" t="s">
+      <c r="J5" s="135"/>
+      <c r="K5" s="142" t="s">
         <v>270</v>
       </c>
-      <c r="L5" s="114"/>
+      <c r="L5" s="143"/>
     </row>
     <row r="6" spans="1:47" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="119" t="s">
+      <c r="A6" s="173" t="s">
         <v>271</v>
       </c>
-      <c r="B6" s="120"/>
-      <c r="C6" s="136" t="s">
+      <c r="B6" s="133"/>
+      <c r="C6" s="132" t="s">
         <v>272</v>
       </c>
-      <c r="D6" s="120"/>
-      <c r="E6" s="136" t="s">
+      <c r="D6" s="133"/>
+      <c r="E6" s="132" t="s">
         <v>273</v>
       </c>
-      <c r="F6" s="120"/>
-      <c r="G6" s="122" t="s">
+      <c r="F6" s="133"/>
+      <c r="G6" s="175" t="s">
         <v>274</v>
       </c>
-      <c r="H6" s="120"/>
-      <c r="I6" s="136" t="s">
+      <c r="H6" s="133"/>
+      <c r="I6" s="132" t="s">
         <v>275</v>
       </c>
-      <c r="J6" s="120"/>
-      <c r="K6" s="159" t="s">
+      <c r="J6" s="133"/>
+      <c r="K6" s="138" t="s">
         <v>276</v>
       </c>
-      <c r="L6" s="160"/>
+      <c r="L6" s="139"/>
       <c r="O6" t="s">
         <v>277</v>
       </c>
@@ -32685,7 +32685,7 @@
       </c>
     </row>
     <row r="8" spans="1:47" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="121" t="s">
+      <c r="A8" s="174" t="s">
         <v>300</v>
       </c>
       <c r="B8" s="101"/>
@@ -33123,7 +33123,7 @@
       </c>
       <c r="Q11" s="23">
         <f ca="1">'Watchlist Ratings'!BM7</f>
-        <v>0.24224417295338063</v>
+        <v>0.28381894079882097</v>
       </c>
       <c r="S11" t="str">
         <f ca="1">'Watchlist Ratings'!B7</f>
@@ -33159,11 +33159,11 @@
       </c>
       <c r="AB11">
         <f ca="1">'Watchlist Ratings'!BL7</f>
-        <v>-4.5069756479004019E-2</v>
+        <v>1.8391612561389437E-2</v>
       </c>
       <c r="AC11">
         <f ca="1">'Watchlist Ratings'!BM7</f>
-        <v>0.24224417295338063</v>
+        <v>0.28381894079882097</v>
       </c>
       <c r="AE11" t="s">
         <v>310</v>
@@ -34513,7 +34513,7 @@
       </c>
     </row>
     <row r="24" spans="1:47" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="167" t="s">
+      <c r="A24" s="145" t="s">
         <v>327</v>
       </c>
       <c r="B24" s="101"/>
@@ -34589,7 +34589,7 @@
     <row r="38" spans="2:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="39" spans="2:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="40" spans="2:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="L40" s="175"/>
+      <c r="L40" s="114"/>
       <c r="M40" s="101"/>
       <c r="N40" s="101"/>
       <c r="O40" s="101"/>
@@ -34606,7 +34606,7 @@
       <c r="Q41" s="57"/>
     </row>
     <row r="42" spans="2:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="J42" s="177"/>
+      <c r="J42" s="118"/>
       <c r="K42" s="101"/>
       <c r="L42" s="101"/>
       <c r="M42" s="101"/>
@@ -34691,7 +34691,7 @@
     <row r="60" spans="1:17" ht="4.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="61" spans="1:17" ht="4.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="62" spans="1:17" ht="4.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A62" s="146" t="s">
+      <c r="A62" s="148" t="s">
         <v>328</v>
       </c>
       <c r="B62" s="101"/>
@@ -34971,27 +34971,27 @@
       </c>
       <c r="C67" s="64">
         <f ca="1">'Watchlist Ratings'!BJ7</f>
-        <v>33.104736501877106</v>
+        <v>45.66736611995114</v>
       </c>
       <c r="D67" s="64">
         <f ca="1">'Watchlist Ratings'!BK7</f>
-        <v>99.279542724768191</v>
+        <v>113.25229463500978</v>
       </c>
       <c r="E67" s="65">
         <f ca="1">'Watchlist Ratings'!BL7</f>
-        <v>-4.5069756479004019E-2</v>
+        <v>1.8391612561389437E-2</v>
       </c>
       <c r="F67" s="65">
         <f ca="1">'Watchlist Ratings'!BM7</f>
-        <v>0.24224417295338063</v>
+        <v>0.28381894079882097</v>
       </c>
       <c r="G67" s="65">
         <f t="shared" ca="1" si="0"/>
-        <v>0.28731392943238465</v>
+        <v>0.26542732823743154</v>
       </c>
       <c r="H67" s="63" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>🟡 HOLD</v>
+        <v>🟢 BUY</v>
       </c>
       <c r="J67" s="63" t="str">
         <f ca="1">'Watchlist Ratings'!B7</f>
@@ -35291,29 +35291,29 @@
       </c>
     </row>
     <row r="72" spans="1:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="164" t="str">
+      <c r="A72" s="144" t="str">
         <f ca="1">'Watchlist Ratings'!B12</f>
         <v>NTO</v>
       </c>
-      <c r="B72" s="165"/>
-      <c r="C72" s="165"/>
-      <c r="D72" s="165"/>
-      <c r="E72" s="165"/>
-      <c r="F72" s="165"/>
-      <c r="G72" s="165"/>
-      <c r="H72" s="165"/>
-      <c r="I72" s="166"/>
-      <c r="J72" s="174" t="str">
+      <c r="B72" s="112"/>
+      <c r="C72" s="112"/>
+      <c r="D72" s="112"/>
+      <c r="E72" s="112"/>
+      <c r="F72" s="112"/>
+      <c r="G72" s="112"/>
+      <c r="H72" s="112"/>
+      <c r="I72" s="113"/>
+      <c r="J72" s="111" t="str">
         <f ca="1">'Watchlist Ratings'!B12</f>
         <v>NTO</v>
       </c>
-      <c r="K72" s="165"/>
-      <c r="L72" s="165"/>
-      <c r="M72" s="165"/>
-      <c r="N72" s="165"/>
-      <c r="O72" s="165"/>
-      <c r="P72" s="165"/>
-      <c r="Q72" s="166"/>
+      <c r="K72" s="112"/>
+      <c r="L72" s="112"/>
+      <c r="M72" s="112"/>
+      <c r="N72" s="112"/>
+      <c r="O72" s="112"/>
+      <c r="P72" s="112"/>
+      <c r="Q72" s="113"/>
     </row>
     <row r="73" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="68" t="str">
@@ -35510,7 +35510,7 @@
       </c>
     </row>
     <row r="76" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A76" s="139" t="s">
+      <c r="A76" s="164" t="s">
         <v>341</v>
       </c>
       <c r="B76" s="101"/>
@@ -35540,23 +35540,23 @@
       </c>
       <c r="C77" s="80">
         <f ca="1">VLOOKUP(A77,'Watchlist Ratings'!$B$4:$BM$71,59,FALSE())</f>
-        <v>13</v>
+        <v>17.5</v>
       </c>
       <c r="D77" s="80">
         <f ca="1">VLOOKUP(A77,'Watchlist Ratings'!$B$4:$BM$71,60,FALSE())</f>
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E77" s="81">
         <f ca="1">VLOOKUP(A77,'Watchlist Ratings'!$B$4:$BM$71,61,FALSE())</f>
-        <v>33.104736501877106</v>
+        <v>45.66736611995114</v>
       </c>
       <c r="F77" s="81">
         <f ca="1">VLOOKUP(A77,'Watchlist Ratings'!$B$4:$BM$71,64,FALSE())</f>
-        <v>0.24224417295338063</v>
+        <v>0.28381894079882097</v>
       </c>
       <c r="G77" s="81">
         <f ca="1">F77-E77</f>
-        <v>-32.862492328923729</v>
+        <v>-45.383547179152316</v>
       </c>
       <c r="H77" s="79" t="str">
         <f ca="1">IF(E77&gt;0,"🟢 BUY",IF(E77&gt;-0.05,"🟡 HOLD","🔴 PASS"))</f>
@@ -35598,127 +35598,127 @@
       <c r="A78" s="131" t="s">
         <v>342</v>
       </c>
-      <c r="B78" s="116"/>
-      <c r="C78" s="115" t="s">
+      <c r="B78" s="120"/>
+      <c r="C78" s="170" t="s">
         <v>343</v>
       </c>
-      <c r="D78" s="116"/>
-      <c r="E78" s="134" t="s">
+      <c r="D78" s="120"/>
+      <c r="E78" s="160" t="s">
         <v>344</v>
       </c>
-      <c r="F78" s="116"/>
-      <c r="G78" s="134" t="s">
+      <c r="F78" s="120"/>
+      <c r="G78" s="160" t="s">
         <v>345</v>
       </c>
-      <c r="H78" s="116"/>
-      <c r="I78" s="111" t="s">
+      <c r="H78" s="120"/>
+      <c r="I78" s="167" t="s">
         <v>346</v>
       </c>
       <c r="J78" s="101"/>
       <c r="K78" s="131" t="s">
         <v>347</v>
       </c>
-      <c r="L78" s="116"/>
+      <c r="L78" s="120"/>
       <c r="M78" s="131" t="s">
         <v>348</v>
       </c>
-      <c r="N78" s="116"/>
+      <c r="N78" s="120"/>
       <c r="O78" s="131" t="s">
         <v>349</v>
       </c>
-      <c r="P78" s="116"/>
+      <c r="P78" s="120"/>
       <c r="Q78" s="82" t="str">
         <f>IF(K78&gt;=8.5,"🟢 ALTO",IF(K78&gt;=7.5,"🟡 MEDIO","🔴 BAJO"))</f>
         <v>🟢 ALTO</v>
       </c>
     </row>
     <row r="79" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A79" s="140" t="str">
+      <c r="A79" s="119" t="str">
         <f ca="1">INDEX('Watchlist Ratings'!B:B,MATCH(MAX('Watchlist Ratings'!AN:AN),'Watchlist Ratings'!AN:AN,0))</f>
         <v>CSU</v>
       </c>
-      <c r="B79" s="116"/>
-      <c r="C79" s="168" t="str">
+      <c r="B79" s="120"/>
+      <c r="C79" s="121" t="str">
         <f ca="1">INDEX('Watchlist Ratings'!B:B,MATCH(MAX('Watchlist Ratings'!BM:BM),'Watchlist Ratings'!BM:BM,0))</f>
         <v>KSPI</v>
       </c>
-      <c r="D79" s="116"/>
-      <c r="E79" s="141" t="str">
+      <c r="D79" s="120"/>
+      <c r="E79" s="122" t="str">
         <f ca="1">INDEX('Watchlist Ratings'!B:B,MATCH(MAX('Watchlist Ratings'!BC:BC),'Watchlist Ratings'!BC:BC,0))</f>
         <v>NVDA</v>
       </c>
-      <c r="F79" s="116"/>
-      <c r="G79" s="141" t="str">
+      <c r="F79" s="120"/>
+      <c r="G79" s="122" t="str">
         <f ca="1">INDEX('Watchlist Ratings'!B:B,MATCH(MAX('Watchlist Ratings'!K:K),'Watchlist Ratings'!K:K,0))</f>
         <v>VEEV</v>
       </c>
-      <c r="H79" s="116"/>
+      <c r="H79" s="120"/>
       <c r="I79" s="152" t="str">
         <f ca="1">INDEX('Watchlist Ratings'!B:B,MATCH(MAX('Watchlist Ratings'!L:L),'Watchlist Ratings'!L:L,0))</f>
         <v>MSFT</v>
       </c>
       <c r="J79" s="101"/>
-      <c r="K79" s="140" t="str">
+      <c r="K79" s="119" t="str">
         <f ca="1">INDEX('Watchlist Ratings'!B:B,MATCH(MAX('Watchlist Ratings'!AM:AM),'Watchlist Ratings'!AM:AM,0))</f>
         <v>DSGX</v>
       </c>
-      <c r="L79" s="116"/>
-      <c r="M79" s="140" t="str">
+      <c r="L79" s="120"/>
+      <c r="M79" s="119" t="str">
         <f t="array" aca="1" ref="M79" ca="1">INDEX('Watchlist Ratings'!B:B,MATCH(MIN('Watchlist Ratings'!AW4:AW64),'Watchlist Ratings'!AW4:AW64,0)+3)</f>
         <v>OTLY</v>
       </c>
-      <c r="N79" s="116"/>
-      <c r="O79" s="140" t="str">
+      <c r="N79" s="120"/>
+      <c r="O79" s="119" t="str">
         <f t="array" aca="1" ref="O79" ca="1">INDEX('Watchlist Ratings'!B:B,MATCH(MAX('Watchlist Ratings'!BM4:BM64-'Watchlist Ratings'!BL4:BL64),'Watchlist Ratings'!BM4:BM64-'Watchlist Ratings'!BL4:BL64,0)+3)</f>
         <v>OTLY</v>
       </c>
-      <c r="P79" s="116"/>
+      <c r="P79" s="120"/>
       <c r="Q79" s="79" t="str">
         <f ca="1">IF(K79&gt;=8.5,"🟢 ALTO",IF(K79&gt;=7.5,"🟡 MEDIO","🔴 BAJO"))</f>
         <v>🟢 ALTO</v>
       </c>
     </row>
     <row r="80" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A80" s="132">
+      <c r="A80" s="158">
         <f>MAX('Watchlist Ratings'!AN:AN)</f>
         <v>8.4499999999999993</v>
       </c>
-      <c r="B80" s="116"/>
-      <c r="C80" s="133">
+      <c r="B80" s="120"/>
+      <c r="C80" s="159">
         <f ca="1">MAX('Watchlist Ratings'!BM:BM)</f>
         <v>0.46183288973934067</v>
       </c>
-      <c r="D80" s="116"/>
-      <c r="E80" s="137">
+      <c r="D80" s="120"/>
+      <c r="E80" s="162">
         <f>MAX('Watchlist Ratings'!BC:BC)</f>
         <v>0.83333333333333326</v>
       </c>
-      <c r="F80" s="116"/>
-      <c r="G80" s="137" t="str">
+      <c r="F80" s="120"/>
+      <c r="G80" s="162" t="str">
         <f>MAX('Watchlist Ratings'!K:K)&amp;"/8"</f>
         <v>8/8</v>
       </c>
-      <c r="H80" s="116"/>
-      <c r="I80" s="170" t="str">
+      <c r="H80" s="120"/>
+      <c r="I80" s="124" t="str">
         <f>MAX('Watchlist Ratings'!L:L)&amp;"/3"</f>
         <v>3/3</v>
       </c>
       <c r="J80" s="101"/>
-      <c r="K80" s="171">
+      <c r="K80" s="125">
         <f>MAX('Watchlist Ratings'!AM:AM)</f>
         <v>8.7100000000000009</v>
       </c>
-      <c r="L80" s="116"/>
-      <c r="M80" s="171" t="str">
+      <c r="L80" s="120"/>
+      <c r="M80" s="125" t="str">
         <f ca="1">MIN('Watchlist Ratings'!AW4:AW64)&amp;"x"</f>
         <v>-18.7185554x</v>
       </c>
-      <c r="N80" s="116"/>
-      <c r="O80" s="171" t="str">
+      <c r="N80" s="120"/>
+      <c r="O80" s="125" t="str">
         <f t="array" aca="1" ref="O80" ca="1">TEXT(MAX('Watchlist Ratings'!BM4:BM64-'Watchlist Ratings'!BL4:BL64),"0.0%")</f>
         <v>249.0%</v>
       </c>
-      <c r="P80" s="116"/>
+      <c r="P80" s="120"/>
       <c r="Q80" s="82" t="str">
         <f>IF(K80&gt;=8.5,"🟢 ALTO",IF(K80&gt;=7.5,"🟡 MEDIO","🔴 BAJO"))</f>
         <v>🟢 ALTO</v>
@@ -35789,7 +35789,7 @@
       </c>
     </row>
     <row r="82" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A82" s="172" t="s">
+      <c r="A82" s="126" t="s">
         <v>350</v>
       </c>
       <c r="B82" s="101"/>
@@ -35897,31 +35897,31 @@
     </row>
     <row r="86" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="87" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A87" s="173" t="s">
+      <c r="A87" s="127" t="s">
         <v>342</v>
       </c>
       <c r="B87" s="101"/>
-      <c r="C87" s="118" t="s">
+      <c r="C87" s="172" t="s">
         <v>343</v>
       </c>
       <c r="D87" s="101"/>
-      <c r="E87" s="169" t="s">
+      <c r="E87" s="123" t="s">
         <v>344</v>
       </c>
       <c r="F87" s="101"/>
-      <c r="G87" s="147" t="s">
+      <c r="G87" s="149" t="s">
         <v>345</v>
       </c>
       <c r="H87" s="101"/>
-      <c r="I87" s="148" t="s">
+      <c r="I87" s="150" t="s">
         <v>346</v>
       </c>
       <c r="J87" s="101"/>
-      <c r="K87" s="117" t="s">
+      <c r="K87" s="171" t="s">
         <v>347</v>
       </c>
       <c r="L87" s="101"/>
-      <c r="M87" s="144" t="s">
+      <c r="M87" s="147" t="s">
         <v>348</v>
       </c>
       <c r="N87" s="101"/>
@@ -35931,7 +35931,7 @@
       <c r="P87" s="101"/>
     </row>
     <row r="88" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A88" s="145" t="str">
+      <c r="A88" s="117" t="str">
         <f ca="1">INDEX('Watchlist Ratings'!B$4:B$71,MATCH(MAX('Watchlist Ratings'!AN$4:AN$71),'Watchlist Ratings'!AN$4:AN$71,0))</f>
         <v>CSU</v>
       </c>
@@ -35941,74 +35941,74 @@
         <v>KSPI</v>
       </c>
       <c r="D88" s="101"/>
-      <c r="E88" s="145" t="str">
+      <c r="E88" s="117" t="str">
         <f ca="1">INDEX('Watchlist Ratings'!B$4:B$71,MATCH(MAX('Watchlist Ratings'!BC$4:BC$71),'Watchlist Ratings'!BC$4:BC$71,0))</f>
         <v>NVDA</v>
       </c>
       <c r="F88" s="101"/>
-      <c r="G88" s="145" t="str">
+      <c r="G88" s="117" t="str">
         <f ca="1">INDEX('Watchlist Ratings'!B$4:B$71,MATCH(MAX('Watchlist Ratings'!K$4:K$71),'Watchlist Ratings'!K$4:K$71,0))</f>
         <v>VEEV</v>
       </c>
       <c r="H88" s="101"/>
-      <c r="I88" s="145" t="str">
+      <c r="I88" s="117" t="str">
         <f ca="1">INDEX('Watchlist Ratings'!B$4:B$71,MATCH(MAX('Watchlist Ratings'!L$4:L$71),'Watchlist Ratings'!L$4:L$71,0))</f>
         <v>MSFT</v>
       </c>
       <c r="J88" s="101"/>
-      <c r="K88" s="145" t="str">
+      <c r="K88" s="117" t="str">
         <f ca="1">INDEX('Watchlist Ratings'!B$4:B$71,MATCH(MAX('Watchlist Ratings'!AM$4:AM$71),'Watchlist Ratings'!AM$4:AM$71,0))</f>
         <v>DSGX</v>
       </c>
       <c r="L88" s="101"/>
-      <c r="M88" s="145" t="str">
+      <c r="M88" s="117" t="str">
         <f t="array" aca="1" ref="M88" ca="1">INDEX('Watchlist Ratings'!B$4:B$64,MATCH(MIN(IF('Watchlist Ratings'!AW$4:AW$64&gt;0,'Watchlist Ratings'!AW$4:AW$64)),IF('Watchlist Ratings'!AW$4:AW$64&gt;0,'Watchlist Ratings'!AW$4:AW$64),0))</f>
         <v>CHKP</v>
       </c>
       <c r="N88" s="101"/>
-      <c r="O88" s="145" t="str">
+      <c r="O88" s="117" t="str">
         <f t="array" aca="1" ref="O88" ca="1">INDEX('Watchlist Ratings'!B$4:B$64,MATCH(MAX('Watchlist Ratings'!BM$4:BM$64-'Watchlist Ratings'!BL$4:BL$64),'Watchlist Ratings'!BM$4:BM$64-'Watchlist Ratings'!BL$4:BL$64,0))</f>
         <v>OTLY</v>
       </c>
       <c r="P88" s="101"/>
     </row>
     <row r="89" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A89" s="143">
+      <c r="A89" s="146">
         <f>MAX('Watchlist Ratings'!AN$4:AN$71)</f>
         <v>8.4499999999999993</v>
       </c>
       <c r="B89" s="101"/>
-      <c r="C89" s="150">
+      <c r="C89" s="116">
         <f ca="1">MAX('Watchlist Ratings'!BM$4:BM$64)</f>
         <v>0.46183288973934067</v>
       </c>
       <c r="D89" s="101"/>
-      <c r="E89" s="150">
+      <c r="E89" s="116">
         <f>MAX('Watchlist Ratings'!BC$4:BC$71)</f>
         <v>0.83333333333333326</v>
       </c>
       <c r="F89" s="101"/>
-      <c r="G89" s="149" t="str">
+      <c r="G89" s="110" t="str">
         <f>MAX('Watchlist Ratings'!K$4:K$71)&amp;"/8"</f>
         <v>8/8</v>
       </c>
       <c r="H89" s="101"/>
-      <c r="I89" s="149" t="str">
+      <c r="I89" s="110" t="str">
         <f>MAX('Watchlist Ratings'!L$4:L$71)&amp;"/3"</f>
         <v>3/3</v>
       </c>
       <c r="J89" s="101"/>
-      <c r="K89" s="176">
+      <c r="K89" s="115">
         <f>MAX('Watchlist Ratings'!AM$4:AM$71)</f>
         <v>8.7100000000000009</v>
       </c>
       <c r="L89" s="101"/>
-      <c r="M89" s="149" t="str">
+      <c r="M89" s="110" t="str">
         <f t="array" aca="1" ref="M89" ca="1">MIN(IF('Watchlist Ratings'!AW$4:AW$64&gt;0,'Watchlist Ratings'!AW$4:AW$64))&amp;"x"</f>
         <v>7.9455641x</v>
       </c>
       <c r="N89" s="101"/>
-      <c r="O89" s="149">
+      <c r="O89" s="110">
         <f t="array" aca="1" ref="O89" ca="1">MAX('Watchlist Ratings'!BM$4:BM$64-'Watchlist Ratings'!BL$4:BL$64)</f>
         <v>2.4903577795625393</v>
       </c>
@@ -36016,7 +36016,7 @@
     </row>
     <row r="90" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="91" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A91" s="110" t="s">
+      <c r="A91" s="166" t="s">
         <v>350</v>
       </c>
       <c r="B91" s="101"/>
@@ -36038,44 +36038,38 @@
     </row>
   </sheetData>
   <mergeCells count="86">
-    <mergeCell ref="I89:J89"/>
-    <mergeCell ref="J72:Q72"/>
-    <mergeCell ref="L40:R40"/>
-    <mergeCell ref="K89:L89"/>
-    <mergeCell ref="C89:D89"/>
-    <mergeCell ref="O88:P88"/>
-    <mergeCell ref="J42:Q42"/>
-    <mergeCell ref="O89:P89"/>
-    <mergeCell ref="A88:B88"/>
-    <mergeCell ref="M79:N79"/>
-    <mergeCell ref="C79:D79"/>
-    <mergeCell ref="K88:L88"/>
-    <mergeCell ref="E79:F79"/>
-    <mergeCell ref="M88:N88"/>
-    <mergeCell ref="E87:F87"/>
-    <mergeCell ref="I80:J80"/>
-    <mergeCell ref="K80:L80"/>
-    <mergeCell ref="A82:Q82"/>
-    <mergeCell ref="A79:B79"/>
-    <mergeCell ref="K79:L79"/>
-    <mergeCell ref="A87:B87"/>
-    <mergeCell ref="M80:N80"/>
-    <mergeCell ref="O80:P80"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="K78:L78"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="A72:I72"/>
-    <mergeCell ref="A24:R24"/>
-    <mergeCell ref="O78:P78"/>
-    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="A91:Q91"/>
+    <mergeCell ref="I78:J78"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="C78:D78"/>
+    <mergeCell ref="K87:L87"/>
+    <mergeCell ref="C87:D87"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A8:L8"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A78:B78"/>
+    <mergeCell ref="M78:N78"/>
+    <mergeCell ref="A80:B80"/>
+    <mergeCell ref="C80:D80"/>
+    <mergeCell ref="E78:F78"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="G78:H78"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="E80:F80"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="G80:H80"/>
+    <mergeCell ref="A76:Q76"/>
+    <mergeCell ref="O79:P79"/>
+    <mergeCell ref="G79:H79"/>
+    <mergeCell ref="A4:B4"/>
     <mergeCell ref="A89:B89"/>
     <mergeCell ref="M87:N87"/>
     <mergeCell ref="G88:H88"/>
@@ -36092,38 +36086,44 @@
     <mergeCell ref="O87:P87"/>
     <mergeCell ref="C88:D88"/>
     <mergeCell ref="E88:F88"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A78:B78"/>
-    <mergeCell ref="M78:N78"/>
-    <mergeCell ref="A80:B80"/>
-    <mergeCell ref="C80:D80"/>
-    <mergeCell ref="E78:F78"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="G78:H78"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E80:F80"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="G80:H80"/>
-    <mergeCell ref="A76:Q76"/>
-    <mergeCell ref="O79:P79"/>
-    <mergeCell ref="G79:H79"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A91:Q91"/>
-    <mergeCell ref="I78:J78"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="C78:D78"/>
-    <mergeCell ref="K87:L87"/>
-    <mergeCell ref="C87:D87"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A8:L8"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="K78:L78"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="A72:I72"/>
+    <mergeCell ref="A24:R24"/>
+    <mergeCell ref="O78:P78"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="A88:B88"/>
+    <mergeCell ref="M79:N79"/>
+    <mergeCell ref="C79:D79"/>
+    <mergeCell ref="K88:L88"/>
+    <mergeCell ref="E79:F79"/>
+    <mergeCell ref="M88:N88"/>
+    <mergeCell ref="E87:F87"/>
+    <mergeCell ref="I80:J80"/>
+    <mergeCell ref="K80:L80"/>
+    <mergeCell ref="A82:Q82"/>
+    <mergeCell ref="A79:B79"/>
+    <mergeCell ref="K79:L79"/>
+    <mergeCell ref="A87:B87"/>
+    <mergeCell ref="M80:N80"/>
+    <mergeCell ref="O80:P80"/>
+    <mergeCell ref="I89:J89"/>
+    <mergeCell ref="J72:Q72"/>
+    <mergeCell ref="L40:R40"/>
+    <mergeCell ref="K89:L89"/>
+    <mergeCell ref="C89:D89"/>
+    <mergeCell ref="O88:P88"/>
+    <mergeCell ref="J42:Q42"/>
+    <mergeCell ref="O89:P89"/>
   </mergeCells>
   <conditionalFormatting sqref="F9:F22">
     <cfRule type="cellIs" dxfId="7" priority="2" operator="greaterThanOrEqual">

</xml_diff>